<commit_message>
fix(medical): workbook model now matches the corrected calculator; preview goldens updated
The xlsx builder still emitted the flat-25% salary-after-CT model. Now:
banded CT with marginal relief over chargeable profit, salary and
employer NIC (15% above GBP 5,000) deducted before CT, matching net
definitions both sides, disclosures for associated companies, EA and
primary NIC. Three workbooks regenerated from the fixed builder; the
regenerated incorporation model verified via openpyxl (banded formula
present, no HP codes). ExcelPreview hardcoded figures re-derived from
the INC-A golden; the headline direction flips from costs GBP 1,973 to
saves GBP 1,276 because the old model overtaxed the company side.
tsc clean, vitest 451/451.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014qDeEjABbveKza768xwLMg
</commit_message>
<xml_diff>
--- a/Medical/web/public/resources/incorporation-private/incorporation-model.xlsx
+++ b/Medical/web/public/resources/incorporation-private/incorporation-model.xlsx
@@ -20,11 +20,17 @@
     <definedName name="NI_UPPER">Rates!$B$6</definedName>
     <definedName name="C4_MAIN">Rates!$B$7</definedName>
     <definedName name="C4_UPPER_RATE">Rates!$B$8</definedName>
-    <definedName name="CT_RATE">Rates!$B$9</definedName>
-    <definedName name="DIV_ALLOWANCE">Rates!$B$10</definedName>
-    <definedName name="DIV_BASIC">Rates!$B$11</definedName>
-    <definedName name="DIV_HIGHER">Rates!$B$12</definedName>
-    <definedName name="DIV_ADDITIONAL">Rates!$B$13</definedName>
+    <definedName name="CT_SMALL">Rates!$B$9</definedName>
+    <definedName name="CT_MAIN">Rates!$B$10</definedName>
+    <definedName name="CT_LOWER">Rates!$B$11</definedName>
+    <definedName name="CT_UPPER">Rates!$B$12</definedName>
+    <definedName name="CT_MARGIN">Rates!$B$13</definedName>
+    <definedName name="EMP_NIC_RATE">Rates!$B$14</definedName>
+    <definedName name="EMP_NIC_THRESHOLD">Rates!$B$15</definedName>
+    <definedName name="DIV_ALLOWANCE">Rates!$B$16</definedName>
+    <definedName name="DIV_BASIC">Rates!$B$17</definedName>
+    <definedName name="DIV_HIGHER">Rates!$B$18</definedName>
+    <definedName name="DIV_ADDITIONAL">Rates!$B$19</definedName>
     <definedName name="In_PrivateIncome">'Your figures'!$B$3</definedName>
     <definedName name="In_Expenses">'Your figures'!$B$4</definedName>
     <definedName name="In_NhsIncome">'Your figures'!$B$5</definedName>
@@ -34,26 +40,29 @@
     <definedName name="ST_IncomeTax">'Your figures'!$B$11</definedName>
     <definedName name="ST_Class4">'Your figures'!$B$12</definedName>
     <definedName name="ST_TotalTax">'Your figures'!$B$13</definedName>
-    <definedName name="LTD_CompanyProfit">'Your figures'!$B$16</definedName>
-    <definedName name="LTD_CT">'Your figures'!$B$17</definedName>
-    <definedName name="LTD_ProfitAfterCT">'Your figures'!$B$18</definedName>
-    <definedName name="LTD_DividendAmount">'Your figures'!$B$19</definedName>
-    <definedName name="LTD_TaxableDividends">'Your figures'!$B$20</definedName>
-    <definedName name="LTD_IncomeBeforeDiv">'Your figures'!$B$21</definedName>
-    <definedName name="LTD_DividendTax">'Your figures'!$B$22</definedName>
-    <definedName name="LTD_NhsIncomeTax">'Your figures'!$B$23</definedName>
-    <definedName name="LTD_TotalTax">'Your figures'!$B$24</definedName>
-    <definedName name="TaxSavings">'Your figures'!$B$27</definedName>
-    <definedName name="SavingsPerMonth">'Your figures'!$B$28</definedName>
+    <definedName name="ST_NetIncome">'Your figures'!$B$14</definedName>
+    <definedName name="LTD_CompanyProfit">'Your figures'!$B$17</definedName>
+    <definedName name="LTD_EmployerNIC">'Your figures'!$B$18</definedName>
+    <definedName name="LTD_ChargeableProfit">'Your figures'!$B$19</definedName>
+    <definedName name="LTD_CT">'Your figures'!$B$20</definedName>
+    <definedName name="LTD_DividendAmount">'Your figures'!$B$21</definedName>
+    <definedName name="LTD_TaxableDividends">'Your figures'!$B$22</definedName>
+    <definedName name="LTD_IncomeBeforeDiv">'Your figures'!$B$23</definedName>
+    <definedName name="LTD_DividendTax">'Your figures'!$B$24</definedName>
+    <definedName name="LTD_PayeIncomeTax">'Your figures'!$B$25</definedName>
+    <definedName name="LTD_TotalTax">'Your figures'!$B$26</definedName>
+    <definedName name="LTD_NetIncome">'Your figures'!$B$27</definedName>
+    <definedName name="TaxSavings">'Your figures'!$B$30</definedName>
+    <definedName name="SavingsPerMonth">'Your figures'!$B$31</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="97">
-  <si>
-    <t>Locked rates: do not edit (2026/27 basis, verified 26 August 2026; CT 25% flat in this model: see notes)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="114">
+  <si>
+    <t>Locked rates: do not edit (2026/27 basis, verified 1 September 2026)</t>
   </si>
   <si>
     <t>Income tax: personal allowance (GBP): 2026/27</t>
@@ -77,7 +86,25 @@
     <t>Class 4 NIC: upper rate 2%: 2026/27</t>
   </si>
   <si>
-    <t>Corporation tax: flat 25% (model simplification; see Notes for true bands): F2</t>
+    <t>Corporation tax: small profits rate 19%, profits up to GBP50,000 (CTA 2010 Part 3)</t>
+  </si>
+  <si>
+    <t>Corporation tax: main rate 25%, profits GBP250,000 and above (CTA 2010 Part 3)</t>
+  </si>
+  <si>
+    <t>Corporation tax: small profits limit (GBP)</t>
+  </si>
+  <si>
+    <t>Corporation tax: main rate threshold (GBP)</t>
+  </si>
+  <si>
+    <t>Corporation tax: marginal relief fraction 3/200, between the two limits</t>
+  </si>
+  <si>
+    <t>Employer secondary Class 1 NIC: 15%, from 6 April 2025</t>
+  </si>
+  <si>
+    <t>Employer secondary Class 1 NIC: secondary threshold (GBP)</t>
   </si>
   <si>
     <t>Dividend allowance (GBP): from 6 April 2026 (FA 2026 s.4)</t>
@@ -116,7 +143,7 @@
     <t>Expenses</t>
   </si>
   <si>
-    <t>Corporation tax (25%)</t>
+    <t>Employer NIC</t>
   </si>
   <si>
     <t>Your NHS (PAYE) income for the year (GBP)</t>
@@ -125,7 +152,7 @@
     <t>NHS income</t>
   </si>
   <si>
-    <t>Profit after CT</t>
+    <t>Chargeable profit (after salary and employer NIC)</t>
   </si>
   <si>
     <t>Director salary from the company (GBP)</t>
@@ -134,6 +161,9 @@
     <t>Practice profit</t>
   </si>
   <si>
+    <t>Corporation tax (19% to 25%)</t>
+  </si>
+  <si>
     <t>Director salary</t>
   </si>
   <si>
@@ -158,12 +188,15 @@
     <t>Total tax and NIC</t>
   </si>
   <si>
-    <t>NHS income tax</t>
+    <t>PAYE income tax (NHS + salary)</t>
   </si>
   <si>
     <t>Income tax (GBP)</t>
   </si>
   <si>
+    <t>Net income</t>
+  </si>
+  <si>
     <t>Total tax</t>
   </si>
   <si>
@@ -173,16 +206,22 @@
     <t>Total tax and NIC (GBP)</t>
   </si>
   <si>
+    <t>Net income after tax (GBP)</t>
+  </si>
+  <si>
     <t>Tax saving (negative = incorporating costs more)</t>
   </si>
   <si>
-    <t>Company profit before CT (GBP)</t>
-  </si>
-  <si>
-    <t>Corporation tax at 25% flat (GBP, F2: see Notes)</t>
-  </si>
-  <si>
-    <t>Profit after corporation tax (GBP)</t>
+    <t>Company profit before salary and tax (GBP)</t>
+  </si>
+  <si>
+    <t>Employer NIC on director salary (GBP)</t>
+  </si>
+  <si>
+    <t>Profit chargeable to corporation tax (GBP)</t>
+  </si>
+  <si>
+    <t>Corporation tax (GBP, 19% to 25% with marginal relief)</t>
   </si>
   <si>
     <t>Available dividends (GBP)</t>
@@ -197,7 +236,7 @@
     <t>Dividend tax (GBP)</t>
   </si>
   <si>
-    <t>NHS income tax (PAYE side, GBP)</t>
+    <t>PAYE income tax on NHS + salary (GBP)</t>
   </si>
   <si>
     <t>Limited company total tax (GBP)</t>
@@ -221,7 +260,7 @@
     <t>See Notes</t>
   </si>
   <si>
-    <t>Company dividends are not NHS pensionable, so incorporated private income loses NHS accrual (HP section 2.C).</t>
+    <t>Company dividends are not NHS pensionable, so incorporated private income loses NHS accrual.</t>
   </si>
   <si>
     <t>Private practice incorporation comparison model</t>
@@ -239,7 +278,7 @@
     <t>trader versus through a limited company, on the same income, using 2026/27 income</t>
   </si>
   <si>
-    <t>tax, Class 4 NIC and dividend tax rates.</t>
+    <t>tax, Class 4 NIC, employer NIC, corporation tax and dividend tax rates.</t>
   </si>
   <si>
     <t>How to use:</t>
@@ -275,7 +314,7 @@
     <t>Assumptions and limitations</t>
   </si>
   <si>
-    <t>IMPORTANT: NHS Pension (HP section 2.C)</t>
+    <t>IMPORTANT: NHS Pension</t>
   </si>
   <si>
     <t>Company dividends are NOT NHS pensionable. A limited company cannot hold a GMS or PMS</t>
@@ -290,31 +329,58 @@
     <t>model both sides before deciding.</t>
   </si>
   <si>
-    <t>F2: Corporation tax simplification</t>
-  </si>
-  <si>
-    <t>This model uses CT 25% flat (matching the online calculator). The true CT regime is:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - 19% on profits up to GBP50,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - Marginal relief between GBP50,000 and GBP250,000 (effective ~26.5%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - 25% on profits above GBP250,000</t>
-  </si>
-  <si>
-    <t>The simplification overstates CT for practices with profits below GBP250,000 and thus</t>
-  </si>
-  <si>
-    <t>understates the sole-trader advantage slightly. Speak to a specialist for the true position.</t>
-  </si>
-  <si>
-    <t>Income tax: 2026/27 rates, verified at gov.uk on 26 August 2026 and unchanged from</t>
-  </si>
-  <si>
-    <t>2025/26. PA GBP12,570; basic 20% to GBP50,270; higher 40% to GBP125,140; 45% above.</t>
+    <t>Corporation tax</t>
+  </si>
+  <si>
+    <t>This model charges the real CTA 2010 Part 3 bands: 19% on profits up to GBP50,000,</t>
+  </si>
+  <si>
+    <t>25% on profits at GBP250,000 and above, and marginal relief in between (fraction 3/200).</t>
+  </si>
+  <si>
+    <t>Director salary and employer NIC are deducted from company profit before corporation</t>
+  </si>
+  <si>
+    <t>tax, because both are deductible expenses of the company.</t>
+  </si>
+  <si>
+    <t>Employer National Insurance</t>
+  </si>
+  <si>
+    <t>Employer secondary Class 1 NIC is charged at 15% on director salary above the GBP5,000</t>
+  </si>
+  <si>
+    <t>secondary threshold, from 6 April 2025. No Employment Allowance is applied: a company</t>
+  </si>
+  <si>
+    <t>whose only employee is a single director cannot claim it.</t>
+  </si>
+  <si>
+    <t>Not modelled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Associated companies. The GBP50,000 and GBP250,000 corporation tax limits are not</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    divided between associated companies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Employment Allowance is not applied (see above).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Employee primary Class 1 NIC on the director salary is not modelled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Company running costs, accountancy fees and year-1 incorporation costs.</t>
+  </si>
+  <si>
+    <t>These reduce the advantage of incorporating further.</t>
+  </si>
+  <si>
+    <t>Income tax: 2026/27 rates, verified 1 September 2026 and unchanged from 2025/26.</t>
+  </si>
+  <si>
+    <t>PA GBP12,570; basic 20% to GBP50,270; higher 40% to GBP125,140; 45% above.</t>
   </si>
   <si>
     <t>Class 4 NIC: 6% on sole-trader private practice profit between GBP12,570 and GBP50,270,</t>
@@ -333,12 +399,6 @@
   </si>
   <si>
     <t>after the year end is charged at 35.75% (from 6 April 2026). Repayable under s.458.</t>
-  </si>
-  <si>
-    <t>The model does not include employer NIC on the director's salary, company running costs,</t>
-  </si>
-  <si>
-    <t>accountancy fees or the year-1 incorporation costs. These reduce the advantage further.</t>
   </si>
   <si>
     <t>This is a directional model. Speak to a specialist for your exact position.</t>
@@ -808,7 +868,7 @@
   <sheetPr>
     <tabColor rgb="FF001b3d"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="72" style="1" customWidth="1"/>
@@ -882,31 +942,31 @@
         <v>8</v>
       </c>
       <c r="B9" s="5">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
-        <v>500</v>
+      <c r="B10" s="5">
+        <v>0.25</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="5">
-        <v>0.1075</v>
+      <c r="B11" s="4">
+        <v>50000</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="5">
-        <v>0.3575</v>
+      <c r="B12" s="4">
+        <v>250000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -914,6 +974,54 @@
         <v>12</v>
       </c>
       <c r="B13" s="5">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5">
+        <v>0.1075</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5">
+        <v>0.3575</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5">
         <v>0.3935</v>
       </c>
     </row>
@@ -932,48 +1040,48 @@
   <sheetPr>
     <tabColor rgb="FFb87333"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="4" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B1" s="6"/>
       <c r="D1" s="7" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E1" s="7"/>
       <c r="G1" s="7" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H1" s="7"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B3" s="9">
         <v>100000</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E3" s="10">
         <f>In_PrivateIncome</f>
       </c>
       <c r="G3" s="8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H3" s="10">
         <f>LTD_CompanyProfit</f>
@@ -981,77 +1089,85 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B4" s="9">
         <v>15000</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E4" s="10">
         <f>In_Expenses</f>
       </c>
       <c r="G4" s="8" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H4" s="10">
-        <f>LTD_CT</f>
+        <f>LTD_EmployerNIC</f>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B5" s="9">
         <v>50000</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E5" s="10">
         <f>In_NhsIncome</f>
       </c>
       <c r="G5" s="8" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="H5" s="10">
-        <f>LTD_ProfitAfterCT</f>
+        <f>LTD_ChargeableProfit</f>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B6" s="9">
         <v>12570</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E6" s="12">
         <f>ST_Profit</f>
       </c>
       <c r="G6" s="8" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H6" s="10">
+        <f>LTD_CT</f>
+      </c>
+    </row>
+    <row r="7" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" s="10">
         <f>In_Salary</f>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B8" s="6"/>
       <c r="D8" s="8" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E8" s="10">
         <f>ST_IncomeTax</f>
       </c>
       <c r="G8" s="8" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H8" s="10">
         <f>LTD_DividendAmount</f>
@@ -1059,19 +1175,19 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B9" s="10">
         <f>In_PrivateIncome-In_Expenses</f>
       </c>
       <c r="D9" s="8" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E9" s="10">
         <f>ST_Class4</f>
       </c>
       <c r="G9" s="8" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="H9" s="10">
         <f>LTD_DividendTax</f>
@@ -1079,180 +1195,216 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B10" s="10">
         <f>ST_Profit+In_NhsIncome</f>
       </c>
       <c r="D10" s="11" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E10" s="12">
         <f>ST_TotalTax</f>
       </c>
       <c r="G10" s="8" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H10" s="10">
-        <f>LTD_NhsIncomeTax</f>
+        <f>LTD_PayeIncomeTax</f>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B11" s="10">
         <f>LET(t,MAX(0,ST_TaxableIncome-PA),basic,MIN(t,BRL-PA),higher,IF(t&gt;BRL-PA,MIN(t-(BRL-PA),HRL-BRL),0),additional,IF(t&gt;HRL-PA,t-(HRL-PA),0),basic*0.2+higher*0.4+additional*0.45)</f>
       </c>
+      <c r="D11" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="12">
+        <f>ST_NetIncome</f>
+      </c>
       <c r="G11" s="11" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="H11" s="12">
         <f>LTD_TotalTax</f>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B12" s="10">
         <f>IF(ST_Profit&lt;=NI_LOWER,0,(MIN(ST_Profit,NI_UPPER)-NI_LOWER)*C4_MAIN+MAX(0,ST_Profit-NI_UPPER)*C4_UPPER_RATE)</f>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G12" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="12">
+        <f>LTD_NetIncome</f>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B13" s="14">
         <f>ST_IncomeTax+ST_Class4</f>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="6"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="14">
+        <f>ST_TaxableIncome-ST_TotalTax</f>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="10">
-        <f>In_PrivateIncome-In_Expenses</f>
-      </c>
+      <c r="A16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="6"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B17" s="10">
-        <f>LTD_CompanyProfit*CT_RATE</f>
+        <f>In_PrivateIncome-In_Expenses</f>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B18" s="10">
-        <f>LTD_CompanyProfit-LTD_CT</f>
+        <f>MAX(0,(In_Salary-EMP_NIC_THRESHOLD)*EMP_NIC_RATE)</f>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B19" s="10">
-        <f>LTD_ProfitAfterCT-In_Salary</f>
+        <f>MAX(0,LTD_CompanyProfit-In_Salary-LTD_EmployerNIC)</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B20" s="10">
-        <f>MAX(0,LTD_DividendAmount-DIV_ALLOWANCE)</f>
+        <f>IF(LTD_ChargeableProfit&lt;=CT_LOWER,LTD_ChargeableProfit*CT_SMALL,IF(LTD_ChargeableProfit&gt;=CT_UPPER,LTD_ChargeableProfit*CT_MAIN,LTD_ChargeableProfit*CT_MAIN-CT_MARGIN*(CT_UPPER-LTD_ChargeableProfit)))</f>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B21" s="10">
-        <f>In_NhsIncome+In_Salary</f>
+        <f>LTD_ChargeableProfit-LTD_CT</f>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B22" s="10">
-        <f>IF(LTD_TaxableDividends&lt;=0,0,MIN(LTD_TaxableDividends,MAX(0,BRL-LTD_IncomeBeforeDiv))*DIV_BASIC+MIN(MAX(0,LTD_TaxableDividends-MAX(0,BRL-LTD_IncomeBeforeDiv)),MAX(0,HRL-MAX(LTD_IncomeBeforeDiv,BRL)))*DIV_HIGHER+MAX(0,LTD_TaxableDividends-MAX(0,BRL-LTD_IncomeBeforeDiv)-MAX(0,HRL-MAX(LTD_IncomeBeforeDiv,BRL)))*DIV_ADDITIONAL)</f>
+        <f>MAX(0,LTD_DividendAmount-DIV_ALLOWANCE)</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B23" s="10">
-        <f>LET(t,MAX(0,In_NhsIncome-PA),basic,MIN(t,BRL-PA),higher,IF(t&gt;BRL-PA,MIN(t-(BRL-PA),HRL-BRL),0),additional,IF(t&gt;HRL-PA,t-(HRL-PA),0),basic*0.2+higher*0.4+additional*0.45)</f>
+        <f>In_NhsIncome+In_Salary</f>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B24" s="14">
-        <f>LTD_CT+LTD_DividendTax+LTD_NhsIncomeTax</f>
+      <c r="A24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="10">
+        <f>IF(LTD_TaxableDividends&lt;=0,0,MIN(LTD_TaxableDividends,MAX(0,BRL-LTD_IncomeBeforeDiv))*DIV_BASIC+MIN(MAX(0,LTD_TaxableDividends-MAX(0,BRL-LTD_IncomeBeforeDiv)),MAX(0,HRL-MAX(LTD_IncomeBeforeDiv,BRL)))*DIV_HIGHER+MAX(0,LTD_TaxableDividends-MAX(0,BRL-LTD_IncomeBeforeDiv)-MAX(0,HRL-MAX(LTD_IncomeBeforeDiv,BRL)))*DIV_ADDITIONAL)</f>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="10">
+        <f>LET(t,MAX(0,LTD_IncomeBeforeDiv-PA),basic,MIN(t,BRL-PA),higher,IF(t&gt;BRL-PA,MIN(t-(BRL-PA),HRL-BRL),0),additional,IF(t&gt;HRL-PA,t-(HRL-PA),0),basic*0.2+higher*0.4+additional*0.45)</f>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="6"/>
+      <c r="A26" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="14">
+        <f>LTD_CT+LTD_EmployerNIC+LTD_DividendTax+LTD_PayeIncomeTax</f>
+      </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="12">
+        <v>48</v>
+      </c>
+      <c r="B27" s="14">
+        <f>In_NhsIncome+In_Salary+LTD_DividendAmount-LTD_DividendTax-LTD_PayeIncomeTax</f>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="12">
         <f>ST_TotalTax-LTD_TotalTax</f>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="15">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="15">
         <f>TaxSavings/12</f>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B30">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33">
         <f>IF(ABS(TaxSavings-(ST_TotalTax-LTD_TotalTax))&lt;0.01,"OK","ERROR")</f>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17" t="s">
-        <v>56</v>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1261,9 +1413,9 @@
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="D13:H13"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A29:B29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1283,97 +1435,97 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1384,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -1392,157 +1544,197 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>85</v>
+      <c r="A15" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>88</v>
+      <c r="A20" s="11" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>